<commit_message>
fix: update Attendance.xlsx to reflect recent changes
</commit_message>
<xml_diff>
--- a/Attendance Tracker/Attendance.xlsx
+++ b/Attendance Tracker/Attendance.xlsx
@@ -498,7 +498,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D2" t="n">
         <v>2</v>
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D4" t="n">
         <v>2</v>

</xml_diff>